<commit_message>
somewhat tire fix, for now it manual in using the init positon on Z, added dej and is working as well as MFEval tire model
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/ARTTU.xlsx
+++ b/Scripts_Data/Data_Vehicle/ARTTU.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Main/Develop/Scripts_Data/Data_Vehicle/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Features/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DA83AF4-EF73-7D47-88BD-934E260F22E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{104E1579-6991-E54F-A90A-728F92F2076F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8080" yWindow="1360" windowWidth="25360" windowHeight="18980" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8080" yWindow="1360" windowWidth="25360" windowHeight="18980" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>

</xml_diff>